<commit_message>
Added code for KS statistical analysis
</commit_message>
<xml_diff>
--- a/multi_period_dataset/Final_dataset_info.xlsx
+++ b/multi_period_dataset/Final_dataset_info.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eashw\Desktop\PhD_resesarch\multi-period-MD-RPP-RRV\multi_period_dataset\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_0753421750397D6A206102AB8855B237A12CEDA7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B58168DF-9AF8-47FE-BC96-0C3CB23A1548}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7026" yWindow="4020" windowWidth="17280" windowHeight="9984" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -803,6 +803,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.6"/>
+  <cols>
+    <col min="2" max="9" width="27.296875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="15.6" x14ac:dyDescent="0.6">
       <c r="A1" t="s">

</xml_diff>